<commit_message>
Template: say where a filled-in tech pack goes for a quote
</commit_message>
<xml_diff>
--- a/hln-tech-pack-template.xlsx
+++ b/hln-tech-pack-template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="109">
   <si>
     <t>TECH PACK — COVER</t>
   </si>
@@ -77,6 +77,9 @@
   </si>
   <si>
     <t>US$79</t>
+  </si>
+  <si>
+    <t>Ready to send? Attach this file to a quote request at hlnapparel.com/contact. We reply with a costed quote and a sample plan, usually within five hours.</t>
   </si>
   <si>
     <t>TECH PACK — SKETCH</t>
@@ -347,7 +350,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -379,10 +382,14 @@
     <font>
       <b/>
       <color rgb="FF1F3478"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1F3478"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -392,6 +399,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3478"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8ECF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -512,7 +524,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -527,7 +539,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -875,7 +890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -987,10 +1002,21 @@
         <v>19</v>
       </c>
     </row>
+    <row r="13" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A13:C13"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A13" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1008,12 +1034,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1023,206 +1049,206 @@
       <c r="G2" s="2"/>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="A4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="9"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="10"/>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="9"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="10"/>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="9"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="10"/>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="9"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="10"/>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="9"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="10"/>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="9"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="10"/>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="10"/>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="9"/>
+      <c r="A12" s="8"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="10"/>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="12"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="13"/>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
+      <c r="A15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="9"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="10"/>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="9"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="10"/>
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="9"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="10"/>
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="9"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="10"/>
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="9"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="10"/>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="9"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="10"/>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="9"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="10"/>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="9"/>
+      <c r="A23" s="8"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="10"/>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="10"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="12"/>
+      <c r="A24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="13"/>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B29" s="5"/>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B30" s="5"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B31" s="5"/>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B32" s="5"/>
     </row>
@@ -1255,12 +1281,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1271,28 +1297,28 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1733,12 +1759,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1749,36 +1775,36 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>6</v>
@@ -1802,41 +1828,41 @@
         <v>6</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>6</v>
@@ -1860,12 +1886,12 @@
         <v>6</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>6</v>
@@ -1889,12 +1915,12 @@
         <v>6</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>6</v>
@@ -1918,12 +1944,12 @@
         <v>6</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>6</v>
@@ -1947,12 +1973,12 @@
         <v>6</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>6</v>
@@ -1976,12 +2002,12 @@
         <v>6</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>6</v>
@@ -2005,7 +2031,7 @@
         <v>6</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2029,12 +2055,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2048,7 +2074,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -2056,79 +2082,79 @@
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2207,12 +2233,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2226,7 +2252,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -2234,68 +2260,68 @@
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2374,12 +2400,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2393,7 +2419,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -2401,68 +2427,68 @@
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fillable PDF, garment-type measurements, Spanish and French versions
- PDF: field guide plus a form you can type into in any PDF reader
- Excel: Measurements loads points of measure for eight garment types;
  frozen headers, print setup, BOM example row
- Spanish and French Excel and PDF

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hln-tech-pack-template.xlsx
+++ b/hln-tech-pack-template.xlsx
@@ -11,13 +11,22 @@
     <sheet sheetId="5" name="Construction" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Labels &amp; Packaging" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Colorways" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="POM library" state="hidden" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Cover'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'BOM'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Measurements'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Construction'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Labels &amp; Packaging'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Colorways'!$4:$4</definedName>
+  </definedNames>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="318">
   <si>
     <t>TECH PACK — COVER</t>
   </si>
@@ -97,15 +106,12 @@
     <t>#</t>
   </si>
   <si>
-    <t>Detail</t>
+    <t>Detail — what each number on the sketch means</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>A flat sketch, a clean photo or a marked-up screenshot. Mark seams, pockets, closures and panel breaks.</t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
@@ -118,6 +124,24 @@
     <t>5</t>
   </si>
   <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>e.g. 1: lined hood</t>
+  </si>
+  <si>
     <t>TECH PACK — BILL OF MATERIALS</t>
   </si>
   <si>
@@ -148,18 +172,204 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>e.g. Body</t>
+  </si>
+  <si>
+    <t>French terry</t>
+  </si>
+  <si>
+    <t>80% cotton / 20% polyester</t>
+  </si>
+  <si>
+    <t>320 GSM</t>
+  </si>
+  <si>
+    <t>Pantone 19-4024 TPX</t>
+  </si>
+  <si>
+    <t>swatch sent 12 May</t>
+  </si>
+  <si>
+    <t>1.4 m per piece</t>
+  </si>
+  <si>
+    <t>Enzyme wash, max 5% shrinkage</t>
+  </si>
+  <si>
     <t>TECH PACK — MEASUREMENTS</t>
   </si>
   <si>
     <t>A garment is inspected against this sheet, so it has to be unambiguous. One row per measurement, one column per size, and a tolerance — this is the sheet that prevents a shipment being rejected over a 1 cm difference.</t>
   </si>
   <si>
+    <t>Garment type</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>cm</t>
+  </si>
+  <si>
+    <t>Pick a garment type to load its points of measure, then overwrite any cell. Tolerances are common starting points; agree final values per style.</t>
+  </si>
+  <si>
     <t>Point of measure</t>
   </si>
   <si>
     <t>How it is measured</t>
   </si>
   <si>
+    <t>Tolerance ±</t>
+  </si>
+  <si>
+    <t>TECH PACK — CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>This sheet is where a good sample becomes a repeatable order. Describe the stitches, seams, thread and decoration exactly; anything left vague will be decided by whoever is on the machine.</t>
+  </si>
+  <si>
+    <t>Specification</t>
+  </si>
+  <si>
+    <t>Stitch type and density</t>
+  </si>
+  <si>
+    <t>SNLS 12 SPI</t>
+  </si>
+  <si>
+    <t>Seam type and finish</t>
+  </si>
+  <si>
+    <t>Taped shoulders</t>
+  </si>
+  <si>
+    <t>Thread</t>
+  </si>
+  <si>
+    <t>Tex 30, match body</t>
+  </si>
+  <si>
+    <t>Print position and size</t>
+  </si>
+  <si>
+    <t>Front, 28 × 20 cm, 3 colours</t>
+  </si>
+  <si>
+    <t>Embroidery position and stitches</t>
+  </si>
+  <si>
+    <t>Left chest, ~4,500 stitches</t>
+  </si>
+  <si>
+    <t>Hardware</t>
+  </si>
+  <si>
+    <t>YKK #5, nickel-free</t>
+  </si>
+  <si>
+    <t>Topstitching</t>
+  </si>
+  <si>
+    <t>2 mm, tonal</t>
+  </si>
+  <si>
+    <t>TECH PACK — LABELS &amp; PACKAGING</t>
+  </si>
+  <si>
+    <t>Private label lives here: the trims and print that carry your brand, and the carton the goods arrive in.</t>
+  </si>
+  <si>
+    <t>Main label</t>
+  </si>
+  <si>
+    <t>Woven, centre back</t>
+  </si>
+  <si>
+    <t>Care label</t>
+  </si>
+  <si>
+    <t>EN/ES/FR, side seam</t>
+  </si>
+  <si>
+    <t>Hang tag</t>
+  </si>
+  <si>
+    <t>Matte card, black cord</t>
+  </si>
+  <si>
+    <t>Fold and polybag</t>
+  </si>
+  <si>
+    <t>Tissue wrap, recycled PE bag</t>
+  </si>
+  <si>
+    <t>Barcode or stickers</t>
+  </si>
+  <si>
+    <t>UPC-A</t>
+  </si>
+  <si>
+    <t>Carton packing</t>
+  </si>
+  <si>
+    <t>50 pcs, assorted sizes</t>
+  </si>
+  <si>
+    <t>TECH PACK — COLORWAYS</t>
+  </si>
+  <si>
+    <t>Colour is the most common cause of a bulk-fabric surprise. Name every colour, reference it to something physical and say how many pieces each one carries.</t>
+  </si>
+  <si>
+    <t>Plan</t>
+  </si>
+  <si>
+    <t>Colour name</t>
+  </si>
+  <si>
+    <t>Sea Green</t>
+  </si>
+  <si>
+    <t>Colour reference</t>
+  </si>
+  <si>
+    <t>Pantone 17-5117 TPX</t>
+  </si>
+  <si>
+    <t>Quantity per colour</t>
+  </si>
+  <si>
+    <t>120 / 100 / 80</t>
+  </si>
+  <si>
+    <t>Size breakdown</t>
+  </si>
+  <si>
+    <t>S–XXL, 20% / 30% / 30% / 20%</t>
+  </si>
+  <si>
+    <t>Trim matching</t>
+  </si>
+  <si>
+    <t>Rib and drawcord tonal</t>
+  </si>
+  <si>
+    <t>Repeats and heroes</t>
+  </si>
+  <si>
+    <t>Sea Green is the hero</t>
+  </si>
+  <si>
+    <t>key</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|sizes</t>
+  </si>
+  <si>
     <t>XS</t>
   </si>
   <si>
@@ -178,179 +388,605 @@
     <t>XXL</t>
   </si>
   <si>
-    <t>Tolerance</t>
-  </si>
-  <si>
-    <t>Chest width (2.5 cm below armhole)</t>
-  </si>
-  <si>
-    <t>±1 cm</t>
+    <t>Hoodie / sweatshirt|1</t>
+  </si>
+  <si>
+    <t>Chest width</t>
+  </si>
+  <si>
+    <t>2.5 cm below armhole, laid flat, edge to edge</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|2</t>
   </si>
   <si>
     <t>Body length from HPS</t>
   </si>
   <si>
+    <t>High point shoulder straight down to hem edge</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|3</t>
+  </si>
+  <si>
     <t>Shoulder width</t>
   </si>
   <si>
+    <t>Shoulder seam to shoulder seam, straight across the back</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|4</t>
+  </si>
+  <si>
     <t>Sleeve length from CB</t>
   </si>
   <si>
+    <t>Centre back neck, over the shoulder, to cuff edge</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|5</t>
+  </si>
+  <si>
+    <t>Armhole (straight)</t>
+  </si>
+  <si>
+    <t>Shoulder point straight to underarm seam</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|6</t>
+  </si>
+  <si>
+    <t>Bicep width</t>
+  </si>
+  <si>
+    <t>2.5 cm below armhole, perpendicular to the sleeve fold</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|7</t>
+  </si>
+  <si>
     <t>Hem width (relaxed)</t>
   </si>
   <si>
+    <t>Bottom rib, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|8</t>
+  </si>
+  <si>
     <t>Cuff width (relaxed)</t>
   </si>
   <si>
-    <t>Hood opening</t>
-  </si>
-  <si>
-    <t>Pocket opening / placement</t>
-  </si>
-  <si>
-    <t>TECH PACK — CONSTRUCTION</t>
-  </si>
-  <si>
-    <t>This sheet is where a good sample becomes a repeatable order. Describe the stitches, seams, thread and decoration exactly; anything left vague will be decided by whoever is on the machine.</t>
-  </si>
-  <si>
-    <t>Specification</t>
-  </si>
-  <si>
-    <t>Stitch type and density</t>
-  </si>
-  <si>
-    <t>SNLS 12 SPI</t>
-  </si>
-  <si>
-    <t>Seam type and finish</t>
-  </si>
-  <si>
-    <t>Taped shoulders</t>
-  </si>
-  <si>
-    <t>Thread</t>
-  </si>
-  <si>
-    <t>Tex 30, match body</t>
-  </si>
-  <si>
-    <t>Print position and size</t>
-  </si>
-  <si>
-    <t>Front, 28 × 20 cm, 3 colours</t>
-  </si>
-  <si>
-    <t>Embroidery position and stitches</t>
-  </si>
-  <si>
-    <t>Left chest, ~4,500 stitches</t>
-  </si>
-  <si>
-    <t>Hardware</t>
-  </si>
-  <si>
-    <t>YKK #5, nickel-free</t>
-  </si>
-  <si>
-    <t>Topstitching</t>
-  </si>
-  <si>
-    <t>2 mm, tonal</t>
-  </si>
-  <si>
-    <t>TECH PACK — LABELS &amp; PACKAGING</t>
-  </si>
-  <si>
-    <t>Private label lives here: the trims and print that carry your brand, and the carton the goods arrive in.</t>
-  </si>
-  <si>
-    <t>Main label</t>
-  </si>
-  <si>
-    <t>Woven, centre back</t>
-  </si>
-  <si>
-    <t>Care label</t>
-  </si>
-  <si>
-    <t>EN/ES/FR, side seam</t>
-  </si>
-  <si>
-    <t>Hang tag</t>
-  </si>
-  <si>
-    <t>Matte card, black cord</t>
-  </si>
-  <si>
-    <t>Fold and polybag</t>
-  </si>
-  <si>
-    <t>Tissue wrap, recycled PE bag</t>
-  </si>
-  <si>
-    <t>Barcode or stickers</t>
-  </si>
-  <si>
-    <t>UPC-A</t>
-  </si>
-  <si>
-    <t>Carton packing</t>
-  </si>
-  <si>
-    <t>50 pcs, assorted sizes</t>
-  </si>
-  <si>
-    <t>TECH PACK — COLORWAYS</t>
-  </si>
-  <si>
-    <t>Colour is the most common cause of a bulk-fabric surprise. Name every colour, reference it to something physical and say how many pieces each one carries.</t>
-  </si>
-  <si>
-    <t>Plan</t>
-  </si>
-  <si>
-    <t>Colour name</t>
-  </si>
-  <si>
-    <t>Sea Green</t>
-  </si>
-  <si>
-    <t>Colour reference</t>
-  </si>
-  <si>
-    <t>Pantone 17-5117 TPX</t>
-  </si>
-  <si>
-    <t>Quantity per colour</t>
-  </si>
-  <si>
-    <t>120 / 100 / 80</t>
-  </si>
-  <si>
-    <t>Size breakdown</t>
-  </si>
-  <si>
-    <t>S–XXL, 20% / 30% / 30% / 20%</t>
-  </si>
-  <si>
-    <t>Trim matching</t>
-  </si>
-  <si>
-    <t>Rib and drawcord tonal</t>
-  </si>
-  <si>
-    <t>Repeats and heroes</t>
-  </si>
-  <si>
-    <t>Sea Green is the hero</t>
+    <t>Cuff opening, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|9</t>
+  </si>
+  <si>
+    <t>Hood height</t>
+  </si>
+  <si>
+    <t>Neck seam at HPS to top of hood</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|10</t>
+  </si>
+  <si>
+    <t>Hood width</t>
+  </si>
+  <si>
+    <t>Widest point of the hood, laid flat</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|11</t>
+  </si>
+  <si>
+    <t>Pocket opening</t>
+  </si>
+  <si>
+    <t>Edge to edge along the opening</t>
+  </si>
+  <si>
+    <t>Hoodie / sweatshirt|12</t>
+  </si>
+  <si>
+    <t>Pocket placement</t>
+  </si>
+  <si>
+    <t>From HPS down to pocket top</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|sizes</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|1</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|2</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|3</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|4</t>
+  </si>
+  <si>
+    <t>Sleeve length</t>
+  </si>
+  <si>
+    <t>Shoulder seam to sleeve hem, along the top fold</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|5</t>
+  </si>
+  <si>
+    <t>Sleeve opening</t>
+  </si>
+  <si>
+    <t>Sleeve hem, edge to edge</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|6</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|7</t>
+  </si>
+  <si>
+    <t>Hem width</t>
+  </si>
+  <si>
+    <t>Bottom hem, edge to edge</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|8</t>
+  </si>
+  <si>
+    <t>Neck width</t>
+  </si>
+  <si>
+    <t>Neck seam to neck seam at HPS</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|9</t>
+  </si>
+  <si>
+    <t>Front neck drop</t>
+  </si>
+  <si>
+    <t>HPS line down to front neck seam</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|10</t>
+  </si>
+  <si>
+    <t>Back neck drop</t>
+  </si>
+  <si>
+    <t>HPS line down to back neck seam</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|11</t>
+  </si>
+  <si>
+    <t>Neck rib / collar width</t>
+  </si>
+  <si>
+    <t>Finished rib or collar height at centre back</t>
+  </si>
+  <si>
+    <t>T-shirt / polo|12</t>
+  </si>
+  <si>
+    <t>Placket length (polo)</t>
+  </si>
+  <si>
+    <t>Top of placket to bottom stitch line</t>
+  </si>
+  <si>
+    <t>Jacket|sizes</t>
+  </si>
+  <si>
+    <t>Jacket|1</t>
+  </si>
+  <si>
+    <t>2.5 cm below armhole, zipped, laid flat</t>
+  </si>
+  <si>
+    <t>Jacket|2</t>
+  </si>
+  <si>
+    <t>Body length from CB</t>
+  </si>
+  <si>
+    <t>Centre back neck seam down to hem</t>
+  </si>
+  <si>
+    <t>Jacket|3</t>
+  </si>
+  <si>
+    <t>Jacket|4</t>
+  </si>
+  <si>
+    <t>Jacket|5</t>
+  </si>
+  <si>
+    <t>Jacket|6</t>
+  </si>
+  <si>
+    <t>Jacket|7</t>
+  </si>
+  <si>
+    <t>Cuff opening</t>
+  </si>
+  <si>
+    <t>Cuff, edge to edge, fastened</t>
+  </si>
+  <si>
+    <t>Jacket|8</t>
+  </si>
+  <si>
+    <t>Bottom hem, zipped, edge to edge</t>
+  </si>
+  <si>
+    <t>Jacket|9</t>
+  </si>
+  <si>
+    <t>Collar height at CB</t>
+  </si>
+  <si>
+    <t>Collar seam to collar edge at centre back</t>
+  </si>
+  <si>
+    <t>Jacket|10</t>
+  </si>
+  <si>
+    <t>Front zip length</t>
+  </si>
+  <si>
+    <t>Zip teeth, top stop to bottom stop</t>
+  </si>
+  <si>
+    <t>Jacket|11</t>
+  </si>
+  <si>
+    <t>Pants / joggers|sizes</t>
+  </si>
+  <si>
+    <t>Pants / joggers|1</t>
+  </si>
+  <si>
+    <t>Waist (relaxed)</t>
+  </si>
+  <si>
+    <t>Top of waistband, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Pants / joggers|2</t>
+  </si>
+  <si>
+    <t>Waist (extended)</t>
+  </si>
+  <si>
+    <t>Top of waistband, edge to edge, fully stretched</t>
+  </si>
+  <si>
+    <t>Pants / joggers|3</t>
+  </si>
+  <si>
+    <t>Hip width</t>
+  </si>
+  <si>
+    <t>18 cm below top of waistband, edge to edge</t>
+  </si>
+  <si>
+    <t>Pants / joggers|4</t>
+  </si>
+  <si>
+    <t>Front rise</t>
+  </si>
+  <si>
+    <t>Top of waistband to crotch seam, along the curve</t>
+  </si>
+  <si>
+    <t>Pants / joggers|5</t>
+  </si>
+  <si>
+    <t>Back rise</t>
+  </si>
+  <si>
+    <t>Pants / joggers|6</t>
+  </si>
+  <si>
+    <t>Inseam</t>
+  </si>
+  <si>
+    <t>Crotch seam to hem along the inside leg</t>
+  </si>
+  <si>
+    <t>Pants / joggers|7</t>
+  </si>
+  <si>
+    <t>Outseam</t>
+  </si>
+  <si>
+    <t>Top of waistband to hem along the side</t>
+  </si>
+  <si>
+    <t>Pants / joggers|8</t>
+  </si>
+  <si>
+    <t>Thigh width</t>
+  </si>
+  <si>
+    <t>2.5 cm below crotch, edge to edge</t>
+  </si>
+  <si>
+    <t>Pants / joggers|9</t>
+  </si>
+  <si>
+    <t>Knee width</t>
+  </si>
+  <si>
+    <t>Halfway down the inseam, edge to edge</t>
+  </si>
+  <si>
+    <t>Pants / joggers|10</t>
+  </si>
+  <si>
+    <t>Leg opening</t>
+  </si>
+  <si>
+    <t>Hem or cuff, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Pants / joggers|11</t>
+  </si>
+  <si>
+    <t>Waistband height</t>
+  </si>
+  <si>
+    <t>Finished waistband, top to bottom edge</t>
+  </si>
+  <si>
+    <t>Pants / joggers|12</t>
+  </si>
+  <si>
+    <t>Shorts|sizes</t>
+  </si>
+  <si>
+    <t>Shorts|1</t>
+  </si>
+  <si>
+    <t>Shorts|2</t>
+  </si>
+  <si>
+    <t>Shorts|3</t>
+  </si>
+  <si>
+    <t>Shorts|4</t>
+  </si>
+  <si>
+    <t>Shorts|5</t>
+  </si>
+  <si>
+    <t>Shorts|6</t>
+  </si>
+  <si>
+    <t>Shorts|7</t>
+  </si>
+  <si>
+    <t>Shorts|8</t>
+  </si>
+  <si>
+    <t>Shorts|9</t>
+  </si>
+  <si>
+    <t>Hem, edge to edge</t>
+  </si>
+  <si>
+    <t>Shorts|10</t>
+  </si>
+  <si>
+    <t>Leggings|sizes</t>
+  </si>
+  <si>
+    <t>Leggings|1</t>
+  </si>
+  <si>
+    <t>Leggings|2</t>
+  </si>
+  <si>
+    <t>Leggings|3</t>
+  </si>
+  <si>
+    <t>15 cm below top of waistband, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Leggings|4</t>
+  </si>
+  <si>
+    <t>Leggings|5</t>
+  </si>
+  <si>
+    <t>Leggings|6</t>
+  </si>
+  <si>
+    <t>Leggings|7</t>
+  </si>
+  <si>
+    <t>2.5 cm below crotch, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Leggings|8</t>
+  </si>
+  <si>
+    <t>Halfway down the inseam, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Leggings|9</t>
+  </si>
+  <si>
+    <t>Ankle opening</t>
+  </si>
+  <si>
+    <t>Hem, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Leggings|10</t>
+  </si>
+  <si>
+    <t>Leggings|11</t>
+  </si>
+  <si>
+    <t>Gusset length × width</t>
+  </si>
+  <si>
+    <t>Gusset panel, seam to seam both ways</t>
+  </si>
+  <si>
+    <t>Cap|sizes</t>
+  </si>
+  <si>
+    <t>One size</t>
+  </si>
+  <si>
+    <t>S/M</t>
+  </si>
+  <si>
+    <t>L/XL</t>
+  </si>
+  <si>
+    <t>Cap|1</t>
+  </si>
+  <si>
+    <t>Head circumference</t>
+  </si>
+  <si>
+    <t>Inside the sweatband, at the smallest strap setting</t>
+  </si>
+  <si>
+    <t>Cap|2</t>
+  </si>
+  <si>
+    <t>Crown height</t>
+  </si>
+  <si>
+    <t>Top button to brim seam at centre front</t>
+  </si>
+  <si>
+    <t>Cap|3</t>
+  </si>
+  <si>
+    <t>Brim length</t>
+  </si>
+  <si>
+    <t>Brim seam to brim edge at centre front</t>
+  </si>
+  <si>
+    <t>Cap|4</t>
+  </si>
+  <si>
+    <t>Brim width</t>
+  </si>
+  <si>
+    <t>Widest point of the brim, edge to edge</t>
+  </si>
+  <si>
+    <t>Cap|5</t>
+  </si>
+  <si>
+    <t>Front panel height</t>
+  </si>
+  <si>
+    <t>Brim seam to top button along the front seam</t>
+  </si>
+  <si>
+    <t>Cap|6</t>
+  </si>
+  <si>
+    <t>Back opening</t>
+  </si>
+  <si>
+    <t>Width of the closure opening above the strap</t>
+  </si>
+  <si>
+    <t>Cap|7</t>
+  </si>
+  <si>
+    <t>Strap adjustment range</t>
+  </si>
+  <si>
+    <t>Smallest to largest head circumference the strap allows</t>
+  </si>
+  <si>
+    <t>Socks|sizes</t>
+  </si>
+  <si>
+    <t>Socks|1</t>
+  </si>
+  <si>
+    <t>Foot length</t>
+  </si>
+  <si>
+    <t>Back of heel to toe seam, laid flat</t>
+  </si>
+  <si>
+    <t>Socks|2</t>
+  </si>
+  <si>
+    <t>Leg length</t>
+  </si>
+  <si>
+    <t>Top of heel to top of cuff, laid flat</t>
+  </si>
+  <si>
+    <t>Socks|3</t>
+  </si>
+  <si>
+    <t>Cuff height</t>
+  </si>
+  <si>
+    <t>Finished rib cuff, top to bottom</t>
+  </si>
+  <si>
+    <t>Socks|4</t>
+  </si>
+  <si>
+    <t>Top of cuff, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Socks|5</t>
+  </si>
+  <si>
+    <t>Cuff width (extended)</t>
+  </si>
+  <si>
+    <t>Top of cuff, edge to edge, fully stretched</t>
+  </si>
+  <si>
+    <t>Socks|6</t>
+  </si>
+  <si>
+    <t>Foot width (relaxed)</t>
+  </si>
+  <si>
+    <t>Mid-foot, edge to edge, unstretched</t>
+  </si>
+  <si>
+    <t>Socks|7</t>
+  </si>
+  <si>
+    <t>Heel width</t>
+  </si>
+  <si>
+    <t>Heel pocket, edge to edge</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -387,6 +1023,21 @@
       <b/>
       <color rgb="FF1F3478"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF6B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF6B7280"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1F3478"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -524,7 +1175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -551,6 +1202,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -890,6 +1559,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1017,19 +1689,24 @@
   <hyperlinks>
     <hyperlink ref="A13" r:id="rId1"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;Lhlnapparel.com/tools/tech-pack-template&amp;R&amp;P / &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G32"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
-    <col min="3" max="6" width="18" customWidth="1"/>
+    <col min="2" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1212,61 +1889,174 @@
       <c r="E24" s="12"/>
       <c r="F24" s="13"/>
     </row>
-    <row r="27" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="B29" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="5"/>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
+      <c r="B30" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B30" s="5"/>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
+      <c r="B31" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="5"/>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
+      <c r="B32" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+    </row>
+    <row r="33" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="5"/>
+      <c r="B33" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+    </row>
+    <row r="34" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+    </row>
+    <row r="35" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+    </row>
+    <row r="36" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+    </row>
+    <row r="37" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="14">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="B28:B32"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B37:F37"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="1"/>
+  <headerFooter>
+    <oddFooter>&amp;Lhlnapparel.com/tools/tech-pack-template&amp;R&amp;P / &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H20"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1281,12 +2071,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1297,54 +2087,54 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>6</v>
+      <c r="A5" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1734,6 +2524,32 @@
         <v>6</v>
       </c>
       <c r="H20" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H21" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1741,30 +2557,43 @@
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="A10:A21">
+      <formula1>"Body,Rib,Hood lining,Pocket lining,Drawcord,Zipper,Button / snap,Main label,Care label,Hang tag,Thread,Polybag,Carton"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="A6:A21">
+      <formula1>"Body,Rib,Hood lining,Pocket lining,Drawcord,Zipper,Button / snap,Main label,Care label,Hang tag,Thread,Polybag,Carton"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;Lhlnapparel.com/tools/tech-pack-template&amp;R&amp;P / &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I12"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="8" width="8" customWidth="1"/>
+    <col min="2" max="2" width="44" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1773,278 +2602,536 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
+    <row r="3" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+    </row>
     <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>52</v>
+        <v>64</v>
+      </c>
+      <c r="C4" s="20" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$G$91,MATCH($B$3&amp;"|sizes",'POM library'!$A$2:$A$91,0),1)&amp;"","")</f>
+        <v>XS</v>
+      </c>
+      <c r="D4" s="20" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$G$91,MATCH($B$3&amp;"|sizes",'POM library'!$A$2:$A$91,0),2)&amp;"","")</f>
+        <v>S</v>
+      </c>
+      <c r="E4" s="20" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$G$91,MATCH($B$3&amp;"|sizes",'POM library'!$A$2:$A$91,0),3)&amp;"","")</f>
+        <v>M</v>
+      </c>
+      <c r="F4" s="20" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$G$91,MATCH($B$3&amp;"|sizes",'POM library'!$A$2:$A$91,0),4)&amp;"","")</f>
+        <v>L</v>
+      </c>
+      <c r="G4" s="20" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$G$91,MATCH($B$3&amp;"|sizes",'POM library'!$A$2:$A$91,0),5)&amp;"","")</f>
+        <v>XL</v>
+      </c>
+      <c r="H4" s="20" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$G$91,MATCH($B$3&amp;"|sizes",'POM library'!$A$2:$A$91,0),6)&amp;"","")</f>
+        <v>XXL</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>55</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|1",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Chest width</v>
+      </c>
+      <c r="B5" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|1",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>2.5 cm below armhole, laid flat, edge to edge</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|1",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|2",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Body length from HPS</v>
+      </c>
+      <c r="B6" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|2",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>High point shoulder straight down to hem edge</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I6" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|2",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|3",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Shoulder width</v>
+      </c>
+      <c r="B7" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|3",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Shoulder seam to shoulder seam, straight across the back</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I7" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|3",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|4",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Sleeve length from CB</v>
+      </c>
+      <c r="B8" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|4",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Centre back neck, over the shoulder, to cuff edge</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|4",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|5",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Armhole (straight)</v>
+      </c>
+      <c r="B9" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|5",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Shoulder point straight to underarm seam</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|5",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|6",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Bicep width</v>
+      </c>
+      <c r="B10" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|6",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>2.5 cm below armhole, perpendicular to the sleeve fold</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I10" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|6",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|7",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Hem width (relaxed)</v>
+      </c>
+      <c r="B11" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|7",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Bottom rib, edge to edge, unstretched</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I11" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|7",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|8",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Cuff width (relaxed)</v>
+      </c>
+      <c r="B12" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|8",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Cuff opening, edge to edge, unstretched</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I12" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|8",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|9",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Hood height</v>
+      </c>
+      <c r="B13" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|9",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Neck seam at HPS to top of hood</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G13" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H13" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I13" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|9",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|10",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Hood width</v>
+      </c>
+      <c r="B14" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|10",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Widest point of the hood, laid flat</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I14" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|10",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|11",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Pocket opening</v>
+      </c>
+      <c r="B15" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|11",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Edge to edge along the opening</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G15" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H15" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I15" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|11",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|12",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>Pocket placement</v>
+      </c>
+      <c r="B16" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|12",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>From HPS down to pocket top</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I16" s="21">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|12",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|13",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B17" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|13",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I17" s="21" t="str">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|13",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="str">
+        <f>IFERROR(INDEX('POM library'!$B$2:$B$91,MATCH($B$3&amp;"|14",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v/>
+      </c>
+      <c r="B18" s="5" t="str">
+        <f>IFERROR(INDEX('POM library'!$C$2:$C$91,MATCH($B$3&amp;"|14",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="I18" s="21" t="str">
+        <f>IFERROR(INDEX('POM library'!$D$2:$D$91,MATCH($B$3&amp;"|14",'POM library'!$A$2:$A$91,0)),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="E3:I3"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <dataValidations count="2">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Garment type" error="Pick a garment type from the list, then overwrite any row below." sqref="B3">
+      <formula1>"Hoodie / sweatshirt,T-shirt / polo,Jacket,Pants / joggers,Shorts,Leggings,Cap,Socks"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showErrorMessage="1" sqref="D3">
+      <formula1>"cm,in"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;Lhlnapparel.com/tools/tech-pack-template&amp;R&amp;P / &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2055,12 +3142,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2074,7 +3161,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -2082,79 +3169,79 @@
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2216,13 +3303,19 @@
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;Lhlnapparel.com/tools/tech-pack-template&amp;R&amp;P / &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2233,12 +3326,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2252,7 +3345,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -2260,68 +3353,68 @@
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2383,13 +3476,19 @@
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;Lhlnapparel.com/tools/tech-pack-template&amp;R&amp;P / &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2400,12 +3499,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2419,7 +3518,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>4</v>
@@ -2427,68 +3526,68 @@
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2550,6 +3649,1351 @@
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;Lhlnapparel.com/tools/tech-pack-template&amp;R&amp;P / &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G91"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B7" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7" t="s">
+        <v>134</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" t="s">
+        <v>136</v>
+      </c>
+      <c r="C8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D10">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" t="s">
+        <v>145</v>
+      </c>
+      <c r="C11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>147</v>
+      </c>
+      <c r="B12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" t="s">
+        <v>149</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D13">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>153</v>
+      </c>
+      <c r="B14" t="s">
+        <v>154</v>
+      </c>
+      <c r="C14" t="s">
+        <v>155</v>
+      </c>
+      <c r="D14">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" t="s">
+        <v>118</v>
+      </c>
+      <c r="G15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>157</v>
+      </c>
+      <c r="B16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C16" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B17" t="s">
+        <v>124</v>
+      </c>
+      <c r="C17" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>159</v>
+      </c>
+      <c r="B18" t="s">
+        <v>127</v>
+      </c>
+      <c r="C18" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>160</v>
+      </c>
+      <c r="B19" t="s">
+        <v>161</v>
+      </c>
+      <c r="C19" t="s">
+        <v>162</v>
+      </c>
+      <c r="D19">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>163</v>
+      </c>
+      <c r="B20" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" t="s">
+        <v>165</v>
+      </c>
+      <c r="D20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>166</v>
+      </c>
+      <c r="B21" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21" t="s">
+        <v>134</v>
+      </c>
+      <c r="D21">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>167</v>
+      </c>
+      <c r="B22" t="s">
+        <v>168</v>
+      </c>
+      <c r="C22" t="s">
+        <v>169</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B23" t="s">
+        <v>171</v>
+      </c>
+      <c r="C23" t="s">
+        <v>172</v>
+      </c>
+      <c r="D23">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>173</v>
+      </c>
+      <c r="B24" t="s">
+        <v>174</v>
+      </c>
+      <c r="C24" t="s">
+        <v>175</v>
+      </c>
+      <c r="D24">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B25" t="s">
+        <v>177</v>
+      </c>
+      <c r="C25" t="s">
+        <v>178</v>
+      </c>
+      <c r="D25">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>179</v>
+      </c>
+      <c r="B26" t="s">
+        <v>180</v>
+      </c>
+      <c r="C26" t="s">
+        <v>181</v>
+      </c>
+      <c r="D26">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>182</v>
+      </c>
+      <c r="B27" t="s">
+        <v>183</v>
+      </c>
+      <c r="C27" t="s">
+        <v>184</v>
+      </c>
+      <c r="D27">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>185</v>
+      </c>
+      <c r="B28" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28" t="s">
+        <v>115</v>
+      </c>
+      <c r="D28" t="s">
+        <v>116</v>
+      </c>
+      <c r="E28" t="s">
+        <v>117</v>
+      </c>
+      <c r="F28" t="s">
+        <v>118</v>
+      </c>
+      <c r="G28" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>186</v>
+      </c>
+      <c r="B29" t="s">
+        <v>121</v>
+      </c>
+      <c r="C29" t="s">
+        <v>187</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>188</v>
+      </c>
+      <c r="B30" t="s">
+        <v>189</v>
+      </c>
+      <c r="C30" t="s">
+        <v>190</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>191</v>
+      </c>
+      <c r="B31" t="s">
+        <v>127</v>
+      </c>
+      <c r="C31" t="s">
+        <v>128</v>
+      </c>
+      <c r="D31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>192</v>
+      </c>
+      <c r="B32" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" t="s">
+        <v>131</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>193</v>
+      </c>
+      <c r="B33" t="s">
+        <v>133</v>
+      </c>
+      <c r="C33" t="s">
+        <v>134</v>
+      </c>
+      <c r="D33">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>194</v>
+      </c>
+      <c r="B34" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>195</v>
+      </c>
+      <c r="B35" t="s">
+        <v>196</v>
+      </c>
+      <c r="C35" t="s">
+        <v>197</v>
+      </c>
+      <c r="D35">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>198</v>
+      </c>
+      <c r="B36" t="s">
+        <v>168</v>
+      </c>
+      <c r="C36" t="s">
+        <v>199</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>200</v>
+      </c>
+      <c r="B37" t="s">
+        <v>201</v>
+      </c>
+      <c r="C37" t="s">
+        <v>202</v>
+      </c>
+      <c r="D37">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>203</v>
+      </c>
+      <c r="B38" t="s">
+        <v>204</v>
+      </c>
+      <c r="C38" t="s">
+        <v>205</v>
+      </c>
+      <c r="D38">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>206</v>
+      </c>
+      <c r="B39" t="s">
+        <v>151</v>
+      </c>
+      <c r="C39" t="s">
+        <v>152</v>
+      </c>
+      <c r="D39">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>207</v>
+      </c>
+      <c r="B40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C40" t="s">
+        <v>115</v>
+      </c>
+      <c r="D40" t="s">
+        <v>116</v>
+      </c>
+      <c r="E40" t="s">
+        <v>117</v>
+      </c>
+      <c r="F40" t="s">
+        <v>118</v>
+      </c>
+      <c r="G40" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>208</v>
+      </c>
+      <c r="B41" t="s">
+        <v>209</v>
+      </c>
+      <c r="C41" t="s">
+        <v>210</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>211</v>
+      </c>
+      <c r="B42" t="s">
+        <v>212</v>
+      </c>
+      <c r="C42" t="s">
+        <v>213</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>214</v>
+      </c>
+      <c r="B43" t="s">
+        <v>215</v>
+      </c>
+      <c r="C43" t="s">
+        <v>216</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>217</v>
+      </c>
+      <c r="B44" t="s">
+        <v>218</v>
+      </c>
+      <c r="C44" t="s">
+        <v>219</v>
+      </c>
+      <c r="D44">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>220</v>
+      </c>
+      <c r="B45" t="s">
+        <v>221</v>
+      </c>
+      <c r="C45" t="s">
+        <v>219</v>
+      </c>
+      <c r="D45">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>222</v>
+      </c>
+      <c r="B46" t="s">
+        <v>223</v>
+      </c>
+      <c r="C46" t="s">
+        <v>224</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>225</v>
+      </c>
+      <c r="B47" t="s">
+        <v>226</v>
+      </c>
+      <c r="C47" t="s">
+        <v>227</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>228</v>
+      </c>
+      <c r="B48" t="s">
+        <v>229</v>
+      </c>
+      <c r="C48" t="s">
+        <v>230</v>
+      </c>
+      <c r="D48">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>231</v>
+      </c>
+      <c r="B49" t="s">
+        <v>232</v>
+      </c>
+      <c r="C49" t="s">
+        <v>233</v>
+      </c>
+      <c r="D49">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>234</v>
+      </c>
+      <c r="B50" t="s">
+        <v>235</v>
+      </c>
+      <c r="C50" t="s">
+        <v>236</v>
+      </c>
+      <c r="D50">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>237</v>
+      </c>
+      <c r="B51" t="s">
+        <v>238</v>
+      </c>
+      <c r="C51" t="s">
+        <v>239</v>
+      </c>
+      <c r="D51">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>240</v>
+      </c>
+      <c r="B52" t="s">
+        <v>151</v>
+      </c>
+      <c r="C52" t="s">
+        <v>152</v>
+      </c>
+      <c r="D52">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>241</v>
+      </c>
+      <c r="B53" t="s">
+        <v>114</v>
+      </c>
+      <c r="C53" t="s">
+        <v>115</v>
+      </c>
+      <c r="D53" t="s">
+        <v>116</v>
+      </c>
+      <c r="E53" t="s">
+        <v>117</v>
+      </c>
+      <c r="F53" t="s">
+        <v>118</v>
+      </c>
+      <c r="G53" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>242</v>
+      </c>
+      <c r="B54" t="s">
+        <v>209</v>
+      </c>
+      <c r="C54" t="s">
+        <v>210</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>243</v>
+      </c>
+      <c r="B55" t="s">
+        <v>212</v>
+      </c>
+      <c r="C55" t="s">
+        <v>213</v>
+      </c>
+      <c r="D55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>244</v>
+      </c>
+      <c r="B56" t="s">
+        <v>215</v>
+      </c>
+      <c r="C56" t="s">
+        <v>216</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>245</v>
+      </c>
+      <c r="B57" t="s">
+        <v>218</v>
+      </c>
+      <c r="C57" t="s">
+        <v>219</v>
+      </c>
+      <c r="D57">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>246</v>
+      </c>
+      <c r="B58" t="s">
+        <v>221</v>
+      </c>
+      <c r="C58" t="s">
+        <v>219</v>
+      </c>
+      <c r="D58">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>247</v>
+      </c>
+      <c r="B59" t="s">
+        <v>223</v>
+      </c>
+      <c r="C59" t="s">
+        <v>224</v>
+      </c>
+      <c r="D59">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>248</v>
+      </c>
+      <c r="B60" t="s">
+        <v>226</v>
+      </c>
+      <c r="C60" t="s">
+        <v>227</v>
+      </c>
+      <c r="D60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>249</v>
+      </c>
+      <c r="B61" t="s">
+        <v>229</v>
+      </c>
+      <c r="C61" t="s">
+        <v>230</v>
+      </c>
+      <c r="D61">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>250</v>
+      </c>
+      <c r="B62" t="s">
+        <v>235</v>
+      </c>
+      <c r="C62" t="s">
+        <v>251</v>
+      </c>
+      <c r="D62">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>252</v>
+      </c>
+      <c r="B63" t="s">
+        <v>238</v>
+      </c>
+      <c r="C63" t="s">
+        <v>239</v>
+      </c>
+      <c r="D63">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>253</v>
+      </c>
+      <c r="B64" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" t="s">
+        <v>115</v>
+      </c>
+      <c r="D64" t="s">
+        <v>116</v>
+      </c>
+      <c r="E64" t="s">
+        <v>117</v>
+      </c>
+      <c r="F64" t="s">
+        <v>118</v>
+      </c>
+      <c r="G64" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>254</v>
+      </c>
+      <c r="B65" t="s">
+        <v>209</v>
+      </c>
+      <c r="C65" t="s">
+        <v>210</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>255</v>
+      </c>
+      <c r="B66" t="s">
+        <v>212</v>
+      </c>
+      <c r="C66" t="s">
+        <v>213</v>
+      </c>
+      <c r="D66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>256</v>
+      </c>
+      <c r="B67" t="s">
+        <v>215</v>
+      </c>
+      <c r="C67" t="s">
+        <v>257</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>258</v>
+      </c>
+      <c r="B68" t="s">
+        <v>218</v>
+      </c>
+      <c r="C68" t="s">
+        <v>219</v>
+      </c>
+      <c r="D68">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>259</v>
+      </c>
+      <c r="B69" t="s">
+        <v>221</v>
+      </c>
+      <c r="C69" t="s">
+        <v>219</v>
+      </c>
+      <c r="D69">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>260</v>
+      </c>
+      <c r="B70" t="s">
+        <v>223</v>
+      </c>
+      <c r="C70" t="s">
+        <v>224</v>
+      </c>
+      <c r="D70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>261</v>
+      </c>
+      <c r="B71" t="s">
+        <v>229</v>
+      </c>
+      <c r="C71" t="s">
+        <v>262</v>
+      </c>
+      <c r="D71">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>263</v>
+      </c>
+      <c r="B72" t="s">
+        <v>232</v>
+      </c>
+      <c r="C72" t="s">
+        <v>264</v>
+      </c>
+      <c r="D72">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>265</v>
+      </c>
+      <c r="B73" t="s">
+        <v>266</v>
+      </c>
+      <c r="C73" t="s">
+        <v>267</v>
+      </c>
+      <c r="D73">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>268</v>
+      </c>
+      <c r="B74" t="s">
+        <v>238</v>
+      </c>
+      <c r="C74" t="s">
+        <v>239</v>
+      </c>
+      <c r="D74">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>269</v>
+      </c>
+      <c r="B75" t="s">
+        <v>270</v>
+      </c>
+      <c r="C75" t="s">
+        <v>271</v>
+      </c>
+      <c r="D75">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>272</v>
+      </c>
+      <c r="B76" t="s">
+        <v>273</v>
+      </c>
+      <c r="C76" t="s">
+        <v>274</v>
+      </c>
+      <c r="D76" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>276</v>
+      </c>
+      <c r="B77" t="s">
+        <v>277</v>
+      </c>
+      <c r="C77" t="s">
+        <v>278</v>
+      </c>
+      <c r="D77">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>279</v>
+      </c>
+      <c r="B78" t="s">
+        <v>280</v>
+      </c>
+      <c r="C78" t="s">
+        <v>281</v>
+      </c>
+      <c r="D78">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>282</v>
+      </c>
+      <c r="B79" t="s">
+        <v>283</v>
+      </c>
+      <c r="C79" t="s">
+        <v>284</v>
+      </c>
+      <c r="D79">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>285</v>
+      </c>
+      <c r="B80" t="s">
+        <v>286</v>
+      </c>
+      <c r="C80" t="s">
+        <v>287</v>
+      </c>
+      <c r="D80">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>288</v>
+      </c>
+      <c r="B81" t="s">
+        <v>289</v>
+      </c>
+      <c r="C81" t="s">
+        <v>290</v>
+      </c>
+      <c r="D81">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>291</v>
+      </c>
+      <c r="B82" t="s">
+        <v>292</v>
+      </c>
+      <c r="C82" t="s">
+        <v>293</v>
+      </c>
+      <c r="D82">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>294</v>
+      </c>
+      <c r="B83" t="s">
+        <v>295</v>
+      </c>
+      <c r="C83" t="s">
+        <v>296</v>
+      </c>
+      <c r="D83">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>297</v>
+      </c>
+      <c r="B84" t="s">
+        <v>115</v>
+      </c>
+      <c r="C84" t="s">
+        <v>116</v>
+      </c>
+      <c r="D84" t="s">
+        <v>117</v>
+      </c>
+      <c r="E84" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>298</v>
+      </c>
+      <c r="B85" t="s">
+        <v>299</v>
+      </c>
+      <c r="C85" t="s">
+        <v>300</v>
+      </c>
+      <c r="D85">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>301</v>
+      </c>
+      <c r="B86" t="s">
+        <v>302</v>
+      </c>
+      <c r="C86" t="s">
+        <v>303</v>
+      </c>
+      <c r="D86">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>304</v>
+      </c>
+      <c r="B87" t="s">
+        <v>305</v>
+      </c>
+      <c r="C87" t="s">
+        <v>306</v>
+      </c>
+      <c r="D87">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>307</v>
+      </c>
+      <c r="B88" t="s">
+        <v>142</v>
+      </c>
+      <c r="C88" t="s">
+        <v>308</v>
+      </c>
+      <c r="D88">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>309</v>
+      </c>
+      <c r="B89" t="s">
+        <v>310</v>
+      </c>
+      <c r="C89" t="s">
+        <v>311</v>
+      </c>
+      <c r="D89">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>312</v>
+      </c>
+      <c r="B90" t="s">
+        <v>313</v>
+      </c>
+      <c r="C90" t="s">
+        <v>314</v>
+      </c>
+      <c r="D90">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>315</v>
+      </c>
+      <c r="B91" t="s">
+        <v>316</v>
+      </c>
+      <c r="C91" t="s">
+        <v>317</v>
+      </c>
+      <c r="D91">
+        <v>0.3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>